<commit_message>
Update Function and Manager UI
</commit_message>
<xml_diff>
--- a/Uploads/reports/event_4_participants.xlsx
+++ b/Uploads/reports/event_4_participants.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Event Participants Report</t>
   </si>
@@ -57,24 +57,6 @@
   </si>
   <si>
     <t>Status</t>
-  </si>
-  <si>
-    <t>Kinh Dương Miên</t>
-  </si>
-  <si>
-    <t>kienduong612@gmail.com</t>
-  </si>
-  <si>
-    <t>0123456789</t>
-  </si>
-  <si>
-    <t>APPROVED</t>
-  </si>
-  <si>
-    <t>Nếu Ngày Ấy</t>
-  </si>
-  <si>
-    <t>duongkien12a3@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -141,14 +123,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.8515625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="16.8515625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="26.08203125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.71875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="16.8515625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="16.8515625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.71875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="11.71875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
@@ -215,46 +197,6 @@
       </c>
       <c r="F9" t="s" s="2">
         <v>14</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n" s="0">
-        <v>8.0</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="C10" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="E10" t="n" s="4">
-        <v>45948.996935717594</v>
-      </c>
-      <c r="F10" t="s" s="0">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n" s="0">
-        <v>9.0</v>
-      </c>
-      <c r="B11" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="C11" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="D11" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="E11" t="n" s="4">
-        <v>45949.02218681713</v>
-      </c>
-      <c r="F11" t="s" s="0">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>